<commit_message>
Checking in Day 3 Hearst
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/Hearst/Test.xlsx
+++ b/src/test/resources/TestDriver/Hearst/Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\fyntrac-data\src\test\resources\TestDriver\Hearst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{279E0AF9-2553-46E1-A9CA-8906C0789846}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E70A235-E872-4BD5-9B9B-B0A725F17518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="35">
   <si>
     <t>Steps</t>
   </si>
@@ -126,10 +126,6 @@
     <t>Hearst/ActivityData/CDB_PSD_20251231.xlsx</t>
   </si>
   <si>
-    <t xml:space="preserve">
-DEFERRED_REVENUE</t>
-  </si>
-  <si>
     <t>TOTAL_REVENUE</t>
   </si>
   <si>
@@ -137,6 +133,12 @@
   </si>
   <si>
     <t>Hearst/Model/Hearst_FinalV7.dsl</t>
+  </si>
+  <si>
+    <t>DEFERRED_REVENUE</t>
+  </si>
+  <si>
+    <t>Hearst/ActivityData/CDB_SOD_20260131.xlsx</t>
   </si>
 </sst>
 </file>
@@ -317,7 +319,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -389,7 +391,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -467,6 +469,28 @@
       </c>
       <c r="C13" s="1">
         <v>46022</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="1">
+        <v>46053</v>
       </c>
     </row>
   </sheetData>
@@ -481,7 +505,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.7109375" customWidth="1"/>
@@ -517,12 +541,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>20251231</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C3">
         <v>-2221.4331999999999</v>
@@ -539,7 +563,7 @@
         <v>20251231</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C4">
         <v>-2221.4331999999999</v>
@@ -556,7 +580,7 @@
         <v>20251231</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C5">
         <v>-2221.4331999999999</v>
@@ -566,6 +590,63 @@
       </c>
       <c r="E5">
         <v>-2221.4331999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>20260131</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="4">
+        <v>-12.491199999999999</v>
+      </c>
+      <c r="D6">
+        <f>E3</f>
+        <v>-2221.4331999999999</v>
+      </c>
+      <c r="E6" s="4">
+        <f>D6+C6</f>
+        <v>-2233.9243999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>20260131</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="4">
+        <v>-12.491199999999999</v>
+      </c>
+      <c r="D7">
+        <f>E4</f>
+        <v>-2221.4331999999999</v>
+      </c>
+      <c r="E7" s="4">
+        <f t="shared" ref="E7:E8" si="0">D7+C7</f>
+        <v>-2233.9243999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>20260131</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="4">
+        <v>-12.491199999999999</v>
+      </c>
+      <c r="D8">
+        <f>E5</f>
+        <v>-2221.4331999999999</v>
+      </c>
+      <c r="E8" s="4">
+        <f t="shared" si="0"/>
+        <v>-2233.9243999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checking in hearst updates
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/Hearst/Test.xlsx
+++ b/src/test/resources/TestDriver/Hearst/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\fyntrac-data\src\test\resources\TestDriver\Hearst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E70A235-E872-4BD5-9B9B-B0A725F17518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35733B00-F653-445A-A980-219AE7CC0F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="37">
   <si>
     <t>Steps</t>
   </si>
@@ -139,6 +139,12 @@
   </si>
   <si>
     <t>Hearst/ActivityData/CDB_SOD_20260131.xlsx</t>
+  </si>
+  <si>
+    <t>Hearst/ActivityData/CDB_SOD_20260228.xlsx</t>
+  </si>
+  <si>
+    <t>Hearst/ActivityData/CDB_PSD_20260228.xlsx</t>
   </si>
 </sst>
 </file>
@@ -319,7 +325,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -491,6 +497,39 @@
       </c>
       <c r="C15" s="1">
         <v>46053</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="1">
+        <v>46081</v>
       </c>
     </row>
   </sheetData>
@@ -505,7 +544,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.7109375" customWidth="1"/>
@@ -649,6 +688,63 @@
         <v>-2233.9243999999999</v>
       </c>
     </row>
+    <row r="9" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>20260228</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="4">
+        <v>-4772.7052000000003</v>
+      </c>
+      <c r="D9" s="4">
+        <f>E6</f>
+        <v>-2233.9243999999999</v>
+      </c>
+      <c r="E9" s="4">
+        <f>C9+D9</f>
+        <v>-7006.6296000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>20260228</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="4">
+        <v>-4772.7052000000003</v>
+      </c>
+      <c r="D10" s="4">
+        <f>E7</f>
+        <v>-2233.9243999999999</v>
+      </c>
+      <c r="E10" s="4">
+        <f t="shared" ref="E10:E11" si="1">C10+D10</f>
+        <v>-7006.6296000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>20260228</v>
+      </c>
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="4">
+        <v>-4772.7052000000003</v>
+      </c>
+      <c r="D11" s="4">
+        <f>E8</f>
+        <v>-2233.9243999999999</v>
+      </c>
+      <c r="E11" s="4">
+        <f t="shared" si="1"/>
+        <v>-7006.6296000000002</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.05277777777778" bottom="1.05277777777778" header="0.78750000000000009" footer="0.78750000000000009"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
checking in march file
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/Hearst/Test.xlsx
+++ b/src/test/resources/TestDriver/Hearst/Test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\fyntrac-data\src\test\resources\TestDriver\Hearst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35733B00-F653-445A-A980-219AE7CC0F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6838849D-6F95-475C-83F3-6F1FCED2D075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="39">
   <si>
     <t>Steps</t>
   </si>
@@ -145,6 +145,12 @@
   </si>
   <si>
     <t>Hearst/ActivityData/CDB_PSD_20260228.xlsx</t>
+  </si>
+  <si>
+    <t>Hearst/ActivityData/CDB_SOD_20260331.xlsx</t>
+  </si>
+  <si>
+    <t>Hearst/ActivityData/CDB_PSD_20260331.xlsx</t>
   </si>
 </sst>
 </file>
@@ -325,7 +331,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -530,6 +536,39 @@
       </c>
       <c r="C18" s="1">
         <v>46081</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>7</v>
+      </c>
+      <c r="B20" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="1">
+        <v>46112</v>
       </c>
     </row>
   </sheetData>
@@ -642,7 +681,7 @@
         <v>-12.491199999999999</v>
       </c>
       <c r="D6">
-        <f>E3</f>
+        <f t="shared" ref="D6:D11" si="0">E3</f>
         <v>-2221.4331999999999</v>
       </c>
       <c r="E6" s="4">
@@ -661,11 +700,11 @@
         <v>-12.491199999999999</v>
       </c>
       <c r="D7">
-        <f>E4</f>
+        <f t="shared" si="0"/>
         <v>-2221.4331999999999</v>
       </c>
       <c r="E7" s="4">
-        <f t="shared" ref="E7:E8" si="0">D7+C7</f>
+        <f t="shared" ref="E7:E8" si="1">D7+C7</f>
         <v>-2233.9243999999999</v>
       </c>
     </row>
@@ -680,11 +719,11 @@
         <v>-12.491199999999999</v>
       </c>
       <c r="D8">
-        <f>E5</f>
+        <f t="shared" si="0"/>
         <v>-2221.4331999999999</v>
       </c>
       <c r="E8" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>-2233.9243999999999</v>
       </c>
     </row>
@@ -699,7 +738,7 @@
         <v>-4772.7052000000003</v>
       </c>
       <c r="D9" s="4">
-        <f>E6</f>
+        <f t="shared" si="0"/>
         <v>-2233.9243999999999</v>
       </c>
       <c r="E9" s="4">
@@ -718,11 +757,11 @@
         <v>-4772.7052000000003</v>
       </c>
       <c r="D10" s="4">
-        <f>E7</f>
+        <f t="shared" si="0"/>
         <v>-2233.9243999999999</v>
       </c>
       <c r="E10" s="4">
-        <f t="shared" ref="E10:E11" si="1">C10+D10</f>
+        <f t="shared" ref="E10:E11" si="2">C10+D10</f>
         <v>-7006.6296000000002</v>
       </c>
     </row>
@@ -737,11 +776,11 @@
         <v>-4772.7052000000003</v>
       </c>
       <c r="D11" s="4">
-        <f>E8</f>
+        <f t="shared" si="0"/>
         <v>-2233.9243999999999</v>
       </c>
       <c r="E11" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-7006.6296000000002</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Checking in CDB full
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/Hearst/Test.xlsx
+++ b/src/test/resources/TestDriver/Hearst/Test.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\fyntrac-data\src\test\resources\TestDriver\Hearst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6838849D-6F95-475C-83F3-6F1FCED2D075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2E79FF3-859F-49A6-A27E-53483F6DB1DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test" sheetId="1" r:id="rId1"/>
-    <sheet name="O_Metric" sheetId="8" r:id="rId2"/>
+    <sheet name="x_Metric" sheetId="8" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="47">
   <si>
     <t>Steps</t>
   </si>
@@ -151,6 +151,30 @@
   </si>
   <si>
     <t>Hearst/ActivityData/CDB_PSD_20260331.xlsx</t>
+  </si>
+  <si>
+    <t>Hearst/ActivityData/CDB_SOD_20260430.xlsx</t>
+  </si>
+  <si>
+    <t>Hearst/ActivityData/CDB_PSD_20260430.xlsx</t>
+  </si>
+  <si>
+    <t>Hearst/ActivityData/CDB_SOD_20260531.xlsx</t>
+  </si>
+  <si>
+    <t>Hearst/ActivityData/CDB_PSD_20260531.xlsx</t>
+  </si>
+  <si>
+    <t>Hearst/ActivityData/CDB_SOD_20260731.xlsx</t>
+  </si>
+  <si>
+    <t>Hearst/ActivityData/CDB_PSD_20260731.xlsx</t>
+  </si>
+  <si>
+    <t>Hearst/ActivityData/CDB_SOD_20260630.xlsx</t>
+  </si>
+  <si>
+    <t>Hearst/ActivityData/CDB_PSD_20260630.xlsx</t>
   </si>
 </sst>
 </file>
@@ -331,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -569,6 +593,138 @@
       </c>
       <c r="C21" s="1">
         <v>46112</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>7</v>
+      </c>
+      <c r="B23" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="1">
+        <v>46142</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="1">
+        <v>46173</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>12</v>
+      </c>
+      <c r="B28" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>13</v>
+      </c>
+      <c r="B30" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" s="1">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>7</v>
+      </c>
+      <c r="B32" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" t="s">
+        <v>14</v>
+      </c>
+      <c r="C33" s="1">
+        <v>46234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checking in new model
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/Hearst/Test.xlsx
+++ b/src/test/resources/TestDriver/Hearst/Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\fyntrac-data\src\test\resources\TestDriver\Hearst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E08ABA8-B70F-4FD2-9BF3-DBA29B179DFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13B30890-5106-445D-A726-837065101B0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="57">
   <si>
     <t>Steps</t>
   </si>
@@ -226,6 +226,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -386,7 +387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -602,6 +603,138 @@
       </c>
       <c r="C19" s="1">
         <v>46053</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>7</v>
+      </c>
+      <c r="B21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" s="1">
+        <v>46081</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="1">
+        <v>46112</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>12</v>
+      </c>
+      <c r="B28" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>13</v>
+      </c>
+      <c r="B31" t="s">
+        <v>14</v>
+      </c>
+      <c r="C31" s="1">
+        <v>46142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checking in test case
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDriver/Hearst/Test.xlsx
+++ b/src/test/resources/TestDriver/Hearst/Test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\fyntrac-data\src\test\resources\TestDriver\Hearst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13B30890-5106-445D-A726-837065101B0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B80B788-AAD1-49BE-8933-429A365671E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="57">
   <si>
     <t>Steps</t>
   </si>
@@ -387,7 +387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
@@ -735,6 +735,138 @@
       </c>
       <c r="C31" s="1">
         <v>46142</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B32" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>7</v>
+      </c>
+      <c r="B33" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>13</v>
+      </c>
+      <c r="B35" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="1">
+        <v>46173</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>12</v>
+      </c>
+      <c r="B36" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>7</v>
+      </c>
+      <c r="B37" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>7</v>
+      </c>
+      <c r="B38" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>13</v>
+      </c>
+      <c r="B39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C39" s="1">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>12</v>
+      </c>
+      <c r="B40" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>7</v>
+      </c>
+      <c r="B41" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>7</v>
+      </c>
+      <c r="B42" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>13</v>
+      </c>
+      <c r="B43" t="s">
+        <v>14</v>
+      </c>
+      <c r="C43" s="1">
+        <v>46234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>